<commit_message>
add baseline algo. requirements now holds pip stuff. class notes renamed + moved.
baseline is popularity based on bayesian weighted with number of ratings and avg rating.
</commit_message>
<xml_diff>
--- a/report/model_performance_tracker.xlsx
+++ b/report/model_performance_tracker.xlsx
@@ -1,43 +1,53 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="Лист1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,26 +55,105 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -330,10 +419,108 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>min_ratings</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>test_ratio</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n_recommendations</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>m (percentile)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Hit Rate @10</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Precision @10</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Recall @10</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (Popularity)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>80th pct</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.4468</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.07770000000000001</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0.0351</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Greedy baseline. Recommends same top-10 popular anime to all users. No personalisation.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add BoW, TF-IDF, SVD, Autoencoder, NCF
bag of words, erm frequency–inverse document frequency, singular value decomposition collaborative filtering, autoencoder, neural collaborative filtering. Needs debugging
</commit_message>
<xml_diff>
--- a/report/model_performance_tracker.xlsx
+++ b/report/model_performance_tracker.xlsx
@@ -29,7 +29,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,12 +78,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -424,10 +432,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
@@ -520,6 +528,286 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW vectors, cosine similarity weighted by user rating. No collaborative signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW vectors, cosine similarity weighted by user rating. No collaborative signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW vectors, cosine similarity weighted by user rating. No collaborative signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW vectors, cosine similarity weighted by user rating. No collaborative signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW vectors, cosine similarity weighted by user rating. No collaborative signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.284</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.0451</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Content-based. TF-IDF genre vectors, cosine similarity weighted by user rating. Rare genres weighted higher than common ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0.3515</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0.1852</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Collaborative AE. Dense 128→32→128, Sigmoid output, masked MSE loss. Adam, epochs=20, batch=128, patience=3, train_users=10000.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
implement log for each run. UI in Bulgarian.
I think I have something somewhat runnable and I can start tinkering and logging results.
</commit_message>
<xml_diff>
--- a/report/model_performance_tracker.xlsx
+++ b/report/model_performance_tracker.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Runs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -40,11 +40,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,12 +69,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -447,286 +439,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Run #</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Split</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>min_ratings</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>test_ratio</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>n_recommendations</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>m (percentile)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>epochs</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>batch_size</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>patience</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>embed_dim</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>n_components</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>train_users</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Hit Rate @10</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Precision @10</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Recall @10</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Baseline (Popularity)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>leave-one-out</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>80th pct</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>0.0032</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Greedy baseline. Recommends same top-10 popular anime to all users. No personalisation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>BoW + Cosine Similarity</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>leave-one-out</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0.0015</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Content-based. Genre BoW vectors, cosine similarity weighted by user rating. No collaborative signal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>TF-IDF + Cosine Similarity</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>leave-one-out</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Content-based. TF-IDF genre vectors, cosine similarity weighted by user rating. Rare genres weighted higher than common ones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>SVD Collaborative Filtering</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>leave-one-out</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>0.298</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>0.0298</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>0.298</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Autoencoder</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>leave-one-out</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0.0014</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Collaborative AE. Dense 128→32→128, Sigmoid output, masked MSE loss. Adam, epochs=20, batch=128, patience=3, train_users=10000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>NCF (Neural Collaborative Filtering)</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>leave-one-out</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>User+anime embeddings (32d), concat→Dense64→Dense32→1. MSE loss, Adam, epochs=20, batch=256, patience=3.</t>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>What changed / Comment</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed the matmul error bug. Add run whole pipeline script.
</commit_message>
<xml_diff>
--- a/report/model_performance_tracker.xlsx
+++ b/report/model_performance_tracker.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +40,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,9 +74,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -439,25 +447,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -539,6 +547,686 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>What changed / Comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 21:31</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (Popularity)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Bayesian popularity baseline. m=80th pct. Recommends same top-10 to all users, no personalisation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 21:31</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 21:31</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. TF-IDF genre vectors, L2-normalised. Rare genres weighted higher than common ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 21:31</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 21:31</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Dense 128→32→128, Sigmoid, masked MSE. epochs=20, batch=128, patience=3, train_users=10000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 21:42</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>NCF (Neural Collaborative Filtering)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>User+anime embeddings (32d), concat→Dense64→Dense32→1. MSE loss, Adam. epochs=20, batch=256, patience=3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:01</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:13</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:13</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. TF-IDF genre vectors, L2-normalised. Rare genres weighted higher than common ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:14</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add param controls to UI to test diff values
</commit_message>
<xml_diff>
--- a/report/model_performance_tracker.xlsx
+++ b/report/model_performance_tracker.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -466,6 +466,7 @@
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1230,6 +1231,803 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:33</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (Popularity)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>Bayesian popularity baseline. m=80th pct. Recommends same top-10 to all users, no personalisation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:33</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:33</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. TF-IDF genre vectors, L2-normalised. Rare genres weighted higher than common ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:33</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:34</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Dense 128→32→128, Sigmoid, masked MSE. epochs=20, batch=128, patience=3, train_users=10000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:44</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>NCF (Neural Collaborative Filtering)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>602.5</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>User+anime embeddings (32d), concat→Dense64→Dense32→1. MSE loss, Adam. epochs=20, batch=256, patience=3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:47</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (Popularity)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>Baseline popularity run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:47</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (Popularity)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>Baseline popularity run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:47</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:47</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 22:48</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>SVD n_components=50</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
"final" commit add params on bow and tfidf
At this time we should have some ok-ish comparable runs
</commit_message>
<xml_diff>
--- a/report/model_performance_tracker.xlsx
+++ b/report/model_performance_tracker.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:U68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -457,18 +457,20 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
-    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -509,55 +511,65 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>min_rating_threshold</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>sublinear_tf</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>epochs</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>batch_size</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>patience</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>embed_dim</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>n_components</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>train_users</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Train time (s)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Hit Rate @10</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Precision @10</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Recall @10</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>What changed / Comment</t>
         </is>
@@ -626,16 +638,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O2" s="2" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>0.0032</v>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q2" s="2" t="n">
         <v>0.032</v>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Bayesian popularity baseline. m=80th pct. Recommends same top-10 to all users, no personalisation.</t>
         </is>
@@ -671,10 +693,8 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H3" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -706,16 +726,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O3" s="2" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>0.0015</v>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q3" s="2" t="n">
         <v>0.015</v>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating.</t>
         </is>
@@ -751,14 +781,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>False</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -786,16 +814,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O4" s="2" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>0.002</v>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q4" s="2" t="n">
         <v>0.02</v>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="R4" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>Content-based. TF-IDF genre vectors, L2-normalised. Rare genres weighted higher than common ones.</t>
         </is>
@@ -851,29 +889,39 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="n">
-        <v>0.298</v>
-      </c>
-      <c r="P5" s="2" t="n">
-        <v>0.0298</v>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q5" s="2" t="n">
         <v>0.298</v>
       </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
         </is>
@@ -909,43 +957,53 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="K6" s="2" t="n">
         <v>128</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="L6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>0.0014</v>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q6" s="2" t="n">
         <v>0.014</v>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="R6" s="2" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>Dense 128→32→128, Sigmoid, masked MSE. epochs=20, batch=128, patience=3, train_users=10000.</t>
         </is>
@@ -981,43 +1039,53 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="K7" s="2" t="n">
         <v>256</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="L7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="M7" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O7" s="2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>0.001</v>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q7" s="2" t="n">
         <v>0.01</v>
       </c>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>User+anime embeddings (32d), concat→Dense64→Dense32→1. MSE loss, Adam. epochs=20, batch=256, patience=3.</t>
         </is>
@@ -1053,10 +1121,8 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1088,16 +1154,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O8" s="2" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>0.0015</v>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q8" s="2" t="n">
         <v>0.015</v>
       </c>
-      <c r="R8" s="2" t="inlineStr">
+      <c r="R8" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating.</t>
         </is>
@@ -1133,10 +1209,8 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H9" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1168,16 +1242,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O9" s="2" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="P9" s="2" t="n">
-        <v>0.0015</v>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q9" s="2" t="n">
         <v>0.015</v>
       </c>
-      <c r="R9" s="2" t="inlineStr">
+      <c r="R9" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating.</t>
         </is>
@@ -1213,14 +1297,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>False</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1248,16 +1330,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O10" s="2" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="P10" s="2" t="n">
-        <v>0.002</v>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q10" s="2" t="n">
         <v>0.02</v>
       </c>
-      <c r="R10" s="2" t="inlineStr">
+      <c r="R10" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>Content-based. TF-IDF genre vectors, L2-normalised. Rare genres weighted higher than common ones.</t>
         </is>
@@ -1313,29 +1405,39 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>0.298</v>
-      </c>
-      <c r="P11" s="2" t="n">
-        <v>0.0298</v>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q11" s="2" t="n">
         <v>0.298</v>
       </c>
-      <c r="R11" s="2" t="inlineStr">
+      <c r="R11" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
         <is>
           <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
         </is>
@@ -1404,21 +1506,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O12" s="2" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="P12" s="2" t="n">
-        <v>0.0032</v>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q12" s="2" t="n">
         <v>0.032</v>
       </c>
-      <c r="R12" s="2" t="inlineStr">
+      <c r="R12" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
         <is>
           <t>Bayesian popularity baseline. m=80th pct. Recommends same top-10 to all users, no personalisation.</t>
         </is>
       </c>
-      <c r="S12" s="2" t="n"/>
+      <c r="U12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1450,10 +1562,8 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H13" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -1485,21 +1595,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O13" s="2" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="P13" s="2" t="n">
-        <v>0.0015</v>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q13" s="2" t="n">
         <v>0.015</v>
       </c>
-      <c r="R13" s="2" t="inlineStr">
+      <c r="R13" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
         <is>
           <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating.</t>
         </is>
       </c>
-      <c r="S13" s="2" t="n"/>
+      <c r="U13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1531,14 +1651,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H14" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>False</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1566,21 +1684,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O14" s="2" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="P14" s="2" t="n">
-        <v>0.002</v>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q14" s="2" t="n">
         <v>0.02</v>
       </c>
-      <c r="R14" s="2" t="inlineStr">
+      <c r="R14" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
         <is>
           <t>Content-based. TF-IDF genre vectors, L2-normalised. Rare genres weighted higher than common ones.</t>
         </is>
       </c>
-      <c r="S14" s="2" t="n"/>
+      <c r="U14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1632,32 +1760,42 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="n">
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="n">
         <v>12.6</v>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>0.298</v>
-      </c>
-      <c r="P15" s="2" t="n">
-        <v>0.0298</v>
       </c>
       <c r="Q15" s="2" t="n">
         <v>0.298</v>
       </c>
-      <c r="R15" s="2" t="inlineStr">
+      <c r="R15" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
         <is>
           <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
         </is>
       </c>
-      <c r="S15" s="2" t="n"/>
+      <c r="U15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1689,46 +1827,56 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="K16" s="2" t="n">
         <v>128</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="L16" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="P16" s="2" t="n">
         <v>12.2</v>
-      </c>
-      <c r="O16" s="2" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="P16" s="2" t="n">
-        <v>0.0014</v>
       </c>
       <c r="Q16" s="2" t="n">
         <v>0.014</v>
       </c>
-      <c r="R16" s="2" t="inlineStr">
+      <c r="R16" s="2" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
         <is>
           <t>Dense 128→32→128, Sigmoid, masked MSE. epochs=20, batch=128, patience=3, train_users=10000.</t>
         </is>
       </c>
-      <c r="S16" s="2" t="n"/>
+      <c r="U16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1760,46 +1908,56 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="K17" s="2" t="n">
         <v>256</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="L17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="M17" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="n">
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="n">
         <v>602.5</v>
-      </c>
-      <c r="O17" s="2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="P17" s="2" t="n">
-        <v>0.001</v>
       </c>
       <c r="Q17" s="2" t="n">
         <v>0.01</v>
       </c>
-      <c r="R17" s="2" t="inlineStr">
+      <c r="R17" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
         <is>
           <t>User+anime embeddings (32d), concat→Dense64→Dense32→1. MSE loss, Adam. epochs=20, batch=256, patience=3.</t>
         </is>
       </c>
-      <c r="S17" s="2" t="n"/>
+      <c r="U17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1864,21 +2022,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O18" s="2" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="P18" s="2" t="n">
-        <v>0.0032</v>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q18" s="2" t="n">
         <v>0.032</v>
       </c>
-      <c r="R18" s="2" t="inlineStr">
+      <c r="R18" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run</t>
         </is>
       </c>
-      <c r="S18" s="2" t="n"/>
+      <c r="U18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1943,21 +2111,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O19" s="2" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="P19" s="2" t="n">
-        <v>0.0032</v>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q19" s="2" t="n">
         <v>0.032</v>
       </c>
-      <c r="R19" s="2" t="inlineStr">
+      <c r="R19" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run</t>
         </is>
       </c>
-      <c r="S19" s="2" t="n"/>
+      <c r="U19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1989,10 +2167,8 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H20" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
@@ -2024,21 +2200,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O20" s="2" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="P20" s="2" t="n">
-        <v>0.0015</v>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q20" s="2" t="n">
         <v>0.015</v>
       </c>
-      <c r="R20" s="2" t="inlineStr">
+      <c r="R20" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
         <is>
           <t>BoW cosine run</t>
         </is>
       </c>
-      <c r="S20" s="2" t="n"/>
+      <c r="U20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2070,14 +2256,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="H21" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>False</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2105,21 +2289,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O21" s="2" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="P21" s="2" t="n">
-        <v>0.002</v>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q21" s="2" t="n">
         <v>0.02</v>
       </c>
-      <c r="R21" s="2" t="inlineStr">
+      <c r="R21" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
         <is>
           <t>TF-IDF cosine run</t>
         </is>
       </c>
-      <c r="S21" s="2" t="n"/>
+      <c r="U21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2171,32 +2365,42 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L22" s="2" t="n">
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N22" s="2" t="n">
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="n">
         <v>11.1</v>
-      </c>
-      <c r="O22" s="2" t="n">
-        <v>0.298</v>
-      </c>
-      <c r="P22" s="2" t="n">
-        <v>0.0298</v>
       </c>
       <c r="Q22" s="2" t="n">
         <v>0.298</v>
       </c>
-      <c r="R22" s="2" t="inlineStr">
+      <c r="R22" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
         <is>
           <t>SVD n_components=50</t>
         </is>
       </c>
-      <c r="S22" s="2" t="n"/>
+      <c r="U22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2261,21 +2465,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O23" s="2" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="P23" s="2" t="n">
-        <v>0.0014</v>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q23" s="2" t="n">
         <v>0.014</v>
       </c>
-      <c r="R23" s="2" t="inlineStr">
+      <c r="R23" s="2" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run 50th percentil</t>
         </is>
       </c>
-      <c r="S23" s="2" t="n"/>
+      <c r="U23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2340,21 +2554,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O24" s="2" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="P24" s="2" t="n">
-        <v>0.0016</v>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q24" s="2" t="n">
         <v>0.016</v>
       </c>
-      <c r="R24" s="2" t="inlineStr">
+      <c r="R24" s="2" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run 50th percentil</t>
         </is>
       </c>
-      <c r="S24" s="2" t="n"/>
+      <c r="U24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2419,21 +2643,31 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O25" s="2" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="P25" s="2" t="n">
-        <v>0.0016</v>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q25" s="2" t="n">
         <v>0.016</v>
       </c>
-      <c r="R25" s="2" t="inlineStr">
+      <c r="R25" s="2" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run</t>
         </is>
       </c>
-      <c r="S25" s="2" t="n"/>
+      <c r="U25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2498,16 +2732,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O26" s="2" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="P26" s="2" t="n">
-        <v>0.0054</v>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q26" s="2" t="n">
         <v>0.054</v>
       </c>
-      <c r="R26" s="2" t="inlineStr">
+      <c r="R26" s="2" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="T26" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run 90th percentile</t>
         </is>
@@ -2576,16 +2820,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O27" s="2" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="P27" s="2" t="n">
-        <v>0.0032</v>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q27" s="2" t="n">
         <v>0.032</v>
       </c>
-      <c r="R27" s="2" t="inlineStr">
+      <c r="R27" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run</t>
         </is>
@@ -2654,16 +2908,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O28" s="2" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="P28" s="2" t="n">
-        <v>0.0054</v>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q28" s="2" t="n">
         <v>0.054</v>
       </c>
-      <c r="R28" s="2" t="inlineStr">
+      <c r="R28" s="2" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="T28" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run</t>
         </is>
@@ -2732,16 +2996,26 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O29" s="2" t="n">
-        <v>0.06900000000000001</v>
-      </c>
-      <c r="P29" s="2" t="n">
-        <v>0.0069</v>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q29" s="2" t="n">
         <v>0.06900000000000001</v>
       </c>
-      <c r="R29" s="2" t="inlineStr">
+      <c r="R29" s="2" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="T29" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run</t>
         </is>
@@ -2810,18 +3084,3324 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O30" s="2" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="P30" s="2" t="n">
-        <v>0.0076</v>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q30" s="2" t="n">
         <v>0.076</v>
       </c>
-      <c r="R30" s="2" t="inlineStr">
+      <c r="R30" s="2" t="n">
+        <v>0.0076</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="T30" s="2" t="inlineStr">
         <is>
           <t>Baseline popularity run</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:23</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="R31" s="2" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:25</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:26</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="R33" s="2" t="n">
+        <v>0.0294</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:30</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>0.291</v>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>0.0291</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>0.291</v>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:31</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="S35" s="2" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="T35" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:32</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="Q36" s="2" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="R36" s="2" t="n">
+        <v>0.0271</v>
+      </c>
+      <c r="S36" s="2" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:33</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="R37" s="2" t="n">
+        <v>0.0308</v>
+      </c>
+      <c r="S37" s="2" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:34</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="R38" s="2" t="n">
+        <v>0.0294</v>
+      </c>
+      <c r="S38" s="2" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:35</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>0.314</v>
+      </c>
+      <c r="R39" s="2" t="n">
+        <v>0.0314</v>
+      </c>
+      <c r="S39" s="2" t="n">
+        <v>0.314</v>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:35</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="Q40" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="R40" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="S40" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:37</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="R41" s="2" t="n">
+        <v>0.0303</v>
+      </c>
+      <c r="S41" s="2" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:38</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>0.305</v>
+      </c>
+      <c r="R42" s="2" t="n">
+        <v>0.0305</v>
+      </c>
+      <c r="S42" s="2" t="n">
+        <v>0.305</v>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>SVD run</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:45</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R43" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S43" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:49</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R44" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S44" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:52</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R45" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S45" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:54</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="R46" s="2" t="n">
+        <v>0.0024</v>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:54</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="R47" s="2" t="n">
+        <v>0.0021</v>
+      </c>
+      <c r="S47" s="2" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:54</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="R48" s="2" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:55</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="R49" s="2" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="S49" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:55</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R50" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S50" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:55</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R51" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S51" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:55</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R52" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S52" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:55</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q53" s="2" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="R53" s="2" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="S53" s="2" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="T53" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:56</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R54" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S54" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:59</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I55" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R55" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S55" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T55" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:59</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I56" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R56" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S56" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:59</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I57" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R57" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S57" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T57" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 17:59</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I58" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R58" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S58" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:00</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I59" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q59" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R59" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S59" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:00</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I60" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="R60" s="2" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="S60" s="2" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:01</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="I61" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="R61" s="2" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="S61" s="2" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="T61" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:01</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I62" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="R62" s="2" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="S62" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:01</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I63" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="R63" s="2" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="S63" s="2" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:03</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I64" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q64" s="2" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="R64" s="2" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="S64" s="2" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="T64" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:04</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="I65" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="R65" s="2" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="S65" s="2" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="T65" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:04</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I66" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="R66" s="2" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="S66" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="T66" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF cosine run</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:05</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (Popularity)</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q67" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R67" s="2" t="n">
+        <v>0.0047</v>
+      </c>
+      <c r="S67" s="2" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="T67" s="2" t="inlineStr">
+        <is>
+          <t>Baseline popularity run</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:06</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="R68" s="2" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="S68" s="2" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>BoW cosine run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
another "final" commit. fix bug. add data unzip to run_all and instructions in readme
</commit_message>
<xml_diff>
--- a/report/model_performance_tracker.xlsx
+++ b/report/model_performance_tracker.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U76"/>
+  <dimension ref="A1:U83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7059,6 +7059,566 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:54</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="P77" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q77" s="2" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="R77" s="2" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="S77" s="2" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="T77" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder run</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 18:55</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>512</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="P78" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q78" s="2" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="R78" s="2" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="S78" s="2" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="T78" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder run</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 19:05</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="P79" s="2" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="Q79" s="2" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="R79" s="2" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="S79" s="2" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="T79" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder run</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 19:05</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="P80" s="2" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="Q80" s="2" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="R80" s="2" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="S80" s="2" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="T80" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder run</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 19:11</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="P81" s="2" t="n">
+        <v>265.7</v>
+      </c>
+      <c r="Q81" s="2" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="R81" s="2" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="S81" s="2" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="T81" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder run</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 19:55</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>NCF (Neural Collaborative Filtering)</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="n">
+        <v>2427.4</v>
+      </c>
+      <c r="Q82" s="2" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="R82" s="2" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="S82" s="2" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="T82" s="2" t="inlineStr">
+        <is>
+          <t>NCF run</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 20:28</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>NCF (Neural Collaborative Filtering)</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M83" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P83" s="2" t="n">
+        <v>1011.4</v>
+      </c>
+      <c r="Q83" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R83" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S83" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T83" s="2" t="inlineStr">
+        <is>
+          <t>NCF run</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix major error in autoencoder and NCF.
Both AE and NCF were set up as rating predictors not ranking
</commit_message>
<xml_diff>
--- a/report/model_performance_tracker.xlsx
+++ b/report/model_performance_tracker.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U83"/>
+  <dimension ref="A1:V91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,8 @@
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="40" customWidth="1" min="20" max="20"/>
-    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -574,6 +575,16 @@
           <t>What changed / Comment</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>pairs_per_user</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>n_per_user</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -7617,6 +7628,748 @@
         <is>
           <t>NCF run</t>
         </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 22:49</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (Popularity)</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q84" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="R84" s="2" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="S84" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="T84" s="2" t="inlineStr">
+        <is>
+          <t>Bayesian popularity baseline. m=80th pct. Recommends same top-10 to all users, no personalisation.</t>
+        </is>
+      </c>
+      <c r="U84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V84" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 22:49</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>BoW + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q85" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R85" s="2" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="S85" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="T85" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. Genre BoW, L2-normalised, dot-product cosine. Weighted by user rating. min_rating_threshold=1.</t>
+        </is>
+      </c>
+      <c r="U85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V85" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 22:49</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>TF-IDF + Cosine Similarity</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q86" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R86" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="S86" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T86" s="2" t="inlineStr">
+        <is>
+          <t>Content-based. TF-IDF genre vectors, L2-normalised. sublinear_tf=False, min_rating_threshold=1.</t>
+        </is>
+      </c>
+      <c r="U86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V86" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 22:50</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>SVD Collaborative Filtering</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P87" s="2" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="Q87" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="R87" s="2" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="S87" s="2" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="T87" s="2" t="inlineStr">
+        <is>
+          <t>Collaborative filtering. TruncatedSVD n_components=50. Factorises user-item rating matrix.</t>
+        </is>
+      </c>
+      <c r="U87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V87" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 22:53</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Autoencoder</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K88" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="P88" s="2" t="n">
+        <v>168.6</v>
+      </c>
+      <c r="Q88" s="2" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="R88" s="2" t="n">
+        <v>0.0024</v>
+      </c>
+      <c r="S88" s="2" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="T88" s="2" t="inlineStr">
+        <is>
+          <t>[v2] Dense 128→32→128, Sigmoid, BPR ranking loss. epochs=20, batch=128, patience=3, pairs_per_user=20, train_users=10000.</t>
+        </is>
+      </c>
+      <c r="U88" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="V88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 22:54</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>NCF (Neural Collaborative Filtering)</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K89" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="L89" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M89" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="Q89" s="2" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="R89" s="2" t="n">
+        <v>0.0109</v>
+      </c>
+      <c r="S89" s="2" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="T89" s="2" t="inlineStr">
+        <is>
+          <t>[v2] User+anime embeddings (32d), concat→Dense64→Dense32→1. BPR ranking loss, Adam. epochs=20, batch=256, patience=3, n_per_user=10.</t>
+        </is>
+      </c>
+      <c r="U89" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V89" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 22:57</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>NCF (Neural Collaborative Filtering)</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K90" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="L90" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M90" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="Q90" s="2" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="R90" s="2" t="n">
+        <v>0.0104</v>
+      </c>
+      <c r="S90" s="2" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="T90" s="2" t="inlineStr">
+        <is>
+          <t>NCF v2 run</t>
+        </is>
+      </c>
+      <c r="U90" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V90" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 23:00</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>NCF (Neural Collaborative Filtering)</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>leave-one-out</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K91" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M91" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P91" s="2" t="n">
+        <v>107.9</v>
+      </c>
+      <c r="Q91" s="2" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="R91" s="2" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="S91" s="2" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="T91" s="2" t="inlineStr">
+        <is>
+          <t>NCF v2 run</t>
+        </is>
+      </c>
+      <c r="U91" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V91" s="2" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>